<commit_message>
out-of-competition athletes were messing rankings
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionBook/Score-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionBook/Score-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\competitionBook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B01999-BBE8-4722-92F0-866015037197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1062B15F-0A4E-4219-8D9E-1A149AE939A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="447" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="447" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C" sheetId="35" r:id="rId1"/>
@@ -513,7 +513,7 @@
     <t>${l.categoryScoreRank &lt; 0 ? t.get("Results.Extra/Invited") : (l.categoryScoreRank &gt; 0 ? l.categoryScoreRank : "" )}</t>
   </si>
   <si>
-    <t>${l.categoryScoreRank}</t>
+    <t>${l.categoryScoreRank &lt; 0 ? 0 : l.categoryScoreRank}</t>
   </si>
 </sst>
 </file>
@@ -1489,10 +1489,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1548,6 +1544,10 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -1611,47 +1611,7 @@
     <cellStyle name="Titre 1 1 1" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
     <cellStyle name="Titre de la feuille" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -5513,59 +5473,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="110" t="s">
+      <c r="A1" s="109" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="112" t="s">
+      <c r="B1" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="114" t="s">
+      <c r="C1" s="113" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="116" t="s">
+      <c r="D1" s="115" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="118" t="s">
+      <c r="E1" s="117" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="118" t="s">
+      <c r="F1" s="117" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="118" t="s">
+      <c r="G1" s="117" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="118" t="s">
+      <c r="H1" s="117" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="120" t="s">
+      <c r="I1" s="119" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="120" t="s">
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="119" t="s">
         <v>45</v>
       </c>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-      <c r="R1" s="121"/>
-      <c r="S1" s="106" t="s">
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="105" t="s">
         <v>139</v>
       </c>
-      <c r="T1" s="107"/>
-      <c r="U1" s="108"/>
+      <c r="T1" s="106"/>
+      <c r="U1" s="107"/>
     </row>
     <row r="2" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="111"/>
-      <c r="B2" s="113"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
+      <c r="A2" s="110"/>
+      <c r="B2" s="112"/>
+      <c r="C2" s="114"/>
+      <c r="D2" s="116"/>
+      <c r="E2" s="118"/>
+      <c r="F2" s="118"/>
+      <c r="G2" s="118"/>
+      <c r="H2" s="118"/>
       <c r="I2" s="32">
         <v>1</v>
       </c>
@@ -5801,11 +5761,11 @@
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C15" s="1"/>
-      <c r="R15" s="109"/>
+      <c r="R15" s="108"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C16" s="1"/>
-      <c r="R16" s="109"/>
+      <c r="R16" s="108"/>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C17" s="1"/>
@@ -6096,21 +6056,13 @@
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="N1:R1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:C8">
-    <cfRule type="expression" dxfId="12" priority="4" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B9:C9">
-    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="B8:C9">
+    <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:D4">
-    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6166,59 +6118,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="110" t="s">
+      <c r="A1" s="109" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="112" t="s">
+      <c r="B1" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="114" t="s">
+      <c r="C1" s="113" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="116" t="s">
+      <c r="D1" s="115" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="118" t="s">
+      <c r="E1" s="117" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="118" t="s">
+      <c r="F1" s="117" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="118" t="s">
+      <c r="G1" s="117" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="118" t="s">
+      <c r="H1" s="117" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="120" t="s">
+      <c r="I1" s="119" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="120" t="s">
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="119" t="s">
         <v>45</v>
       </c>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-      <c r="R1" s="121"/>
-      <c r="S1" s="106" t="s">
+      <c r="O1" s="120"/>
+      <c r="P1" s="120"/>
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="105" t="s">
         <v>139</v>
       </c>
-      <c r="T1" s="107"/>
-      <c r="U1" s="108"/>
+      <c r="T1" s="106"/>
+      <c r="U1" s="107"/>
     </row>
     <row r="2" spans="1:23" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="111"/>
-      <c r="B2" s="113"/>
-      <c r="C2" s="115"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
+      <c r="A2" s="110"/>
+      <c r="B2" s="112"/>
+      <c r="C2" s="114"/>
+      <c r="D2" s="116"/>
+      <c r="E2" s="118"/>
+      <c r="F2" s="118"/>
+      <c r="G2" s="118"/>
+      <c r="H2" s="118"/>
       <c r="I2" s="32">
         <v>1</v>
       </c>
@@ -6455,11 +6407,11 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="C16" s="1"/>
-      <c r="P16" s="109"/>
+      <c r="P16" s="108"/>
     </row>
     <row r="17" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C17" s="1"/>
-      <c r="P17" s="109"/>
+      <c r="P17" s="108"/>
     </row>
     <row r="18" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C18" s="1"/>
@@ -6750,21 +6702,13 @@
     <mergeCell ref="I1:M1"/>
     <mergeCell ref="N1:R1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:C8">
-    <cfRule type="expression" dxfId="8" priority="4" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B9:C9">
-    <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="B8:C9">
+    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:D4">
-    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6825,10 +6769,10 @@
       <c r="C1" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="116" t="s">
+      <c r="D1" s="115" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="118" t="s">
+      <c r="E1" s="117" t="s">
         <v>40</v>
       </c>
       <c r="F1" s="127" t="s">
@@ -6855,10 +6799,10 @@
       <c r="Q1" s="132" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="105" t="s">
+      <c r="R1" s="121" t="s">
         <v>140</v>
       </c>
-      <c r="S1" s="105"/>
+      <c r="S1" s="121"/>
       <c r="U1"/>
       <c r="V1"/>
     </row>
@@ -6867,7 +6811,7 @@
       <c r="B2" s="123"/>
       <c r="C2" s="125"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="118"/>
+      <c r="E2" s="117"/>
       <c r="F2" s="127"/>
       <c r="G2" s="128"/>
       <c r="H2" s="130"/>
@@ -7316,7 +7260,7 @@
     <mergeCell ref="Q1:Q2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="expression" dxfId="4" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
       <formula>AND(("$'Hommes Sinclair'.$#REF!$#REF!"),"$'Hommes Sinclair'.$#REF!$#REF!","$'Hommes Sinclair'.$#REF!$#REF!")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7371,10 +7315,10 @@
       <c r="C1" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="116" t="s">
+      <c r="D1" s="115" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="118" t="s">
+      <c r="E1" s="117" t="s">
         <v>40</v>
       </c>
       <c r="F1" s="127" t="s">
@@ -7401,17 +7345,17 @@
       <c r="Q1" s="132" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="105" t="s">
+      <c r="R1" s="121" t="s">
         <v>140</v>
       </c>
-      <c r="S1" s="105"/>
+      <c r="S1" s="121"/>
     </row>
     <row r="2" spans="1:19" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="123"/>
       <c r="B2" s="123"/>
       <c r="C2" s="125"/>
       <c r="D2" s="126"/>
-      <c r="E2" s="118"/>
+      <c r="E2" s="117"/>
       <c r="F2" s="127"/>
       <c r="G2" s="128"/>
       <c r="H2" s="130"/>
@@ -7835,7 +7779,7 @@
     <mergeCell ref="Q1:Q2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
       <formula>AND(("$'Hommes Sinclair'.$#REF!$#REF!"),"$'Hommes Sinclair'.$#REF!$#REF!","$'Hommes Sinclair'.$#REF!$#REF!")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9165,10 +9109,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5:D5">
-    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>